<commit_message>
Outreach: offer free trial (15 days to a month) alongside free study report
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBvzkEqm3wQqXonEiSiA31
</commit_message>
<xml_diff>
--- a/2-pipeline/goa-leads-pipeline-v1.xlsx
+++ b/2-pipeline/goa-leads-pipeline-v1.xlsx
@@ -671,8 +671,8 @@
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Hi SkinCafe Goa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
@@ -746,8 +746,8 @@
       <c r="S3" s="2" t="inlineStr">
         <is>
           <t>Hi Aesthetic DNA team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -821,8 +821,8 @@
       <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Hi Reborn Skin &amp; Hair Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
@@ -896,8 +896,8 @@
       <c r="S5" s="2" t="inlineStr">
         <is>
           <t>Hi Livom Dental &amp; Cosmetic Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
@@ -963,8 +963,8 @@
       <c r="S6" s="2" t="inlineStr">
         <is>
           <t>Hi Skin Smart Solutions team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
@@ -1038,8 +1038,8 @@
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>Hi Smile Craft Goa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
@@ -1113,8 +1113,8 @@
       <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Hi Dr. Naik's Dental Studio / Kids-N-Braces team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
@@ -1192,8 +1192,8 @@
       <c r="S9" s="2" t="inlineStr">
         <is>
           <t>Hi Physiotherapeautics team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
@@ -1271,8 +1271,8 @@
       <c r="S10" s="2" t="inlineStr">
         <is>
           <t>Hi PhysioFox: The Health Studio team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
@@ -1350,8 +1350,8 @@
       <c r="S11" s="2" t="inlineStr">
         <is>
           <t>Hi Physioedge Physiotherapy team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
@@ -1417,8 +1417,8 @@
       <c r="S12" s="2" t="inlineStr">
         <is>
           <t>Hi Bina Punjani Hair Studio team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -1484,8 +1484,8 @@
       <c r="S13" s="2" t="inlineStr">
         <is>
           <t>Hi Scissorbella team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr">
@@ -1551,8 +1551,8 @@
       <c r="S14" s="2" t="inlineStr">
         <is>
           <t>Hi Nail Master Manish team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
@@ -1618,8 +1618,8 @@
       <c r="S15" s="2" t="inlineStr">
         <is>
           <t>Hi Irina Krutik Nail &amp; Beauty Studio team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T15" s="2" t="inlineStr">
@@ -1685,8 +1685,8 @@
       <c r="S16" s="2" t="inlineStr">
         <is>
           <t>Hi Black Pallet Studio team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T16" s="2" t="inlineStr">
@@ -1752,8 +1752,8 @@
       <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Hi Amanora The Beauty Lounge team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
@@ -1827,8 +1827,8 @@
       <c r="S18" s="2" t="inlineStr">
         <is>
           <t>Hi Studio32 Dental team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T18" s="2" t="inlineStr">
@@ -1898,8 +1898,8 @@
       <c r="S19" s="2" t="inlineStr">
         <is>
           <t>Hi Dr. Emerico's Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T19" s="2" t="inlineStr">
@@ -1961,8 +1961,8 @@
       <c r="S20" s="2" t="inlineStr">
         <is>
           <t>Hi Platinum Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
@@ -2024,8 +2024,8 @@
       <c r="S21" s="2" t="inlineStr">
         <is>
           <t>Hi Nebo Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
@@ -2087,8 +2087,8 @@
       <c r="S22" s="2" t="inlineStr">
         <is>
           <t>Hi Charmin' Smile Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
@@ -2150,8 +2150,8 @@
       <c r="S23" s="2" t="inlineStr">
         <is>
           <t>Hi Reflection Dental Care team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T23" s="2" t="inlineStr">
@@ -2213,8 +2213,8 @@
       <c r="S24" s="2" t="inlineStr">
         <is>
           <t>Hi Kenkre Dental Care team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T24" s="2" t="inlineStr">
@@ -2276,8 +2276,8 @@
       <c r="S25" s="2" t="inlineStr">
         <is>
           <t>Hi Alberto Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T25" s="2" t="inlineStr">
@@ -2351,8 +2351,8 @@
       <c r="S26" s="2" t="inlineStr">
         <is>
           <t>Hi Relive Healthcare team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T26" s="2" t="inlineStr">
@@ -2414,8 +2414,8 @@
       <c r="S27" s="2" t="inlineStr">
         <is>
           <t>Hi Sattva Holistic Rehab team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T27" s="2" t="inlineStr">
@@ -2477,8 +2477,8 @@
       <c r="S28" s="2" t="inlineStr">
         <is>
           <t>Hi Pro Active Physiotherapy Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T28" s="2" t="inlineStr">
@@ -2540,8 +2540,8 @@
       <c r="S29" s="2" t="inlineStr">
         <is>
           <t>Hi Wellness Physiotherapy Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T29" s="2" t="inlineStr">
@@ -2603,8 +2603,8 @@
       <c r="S30" s="2" t="inlineStr">
         <is>
           <t>Hi Parul Physiotherapy &amp; Rehab Center team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T30" s="2" t="inlineStr">
@@ -2678,8 +2678,8 @@
       <c r="S31" s="2" t="inlineStr">
         <is>
           <t>Hi SNIP Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T31" s="2" t="inlineStr">
@@ -2745,8 +2745,8 @@
       <c r="S32" s="2" t="inlineStr">
         <is>
           <t>Hi LM Reborn Hair &amp; Beauty Salon team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr">
@@ -2812,8 +2812,8 @@
       <c r="S33" s="2" t="inlineStr">
         <is>
           <t>Hi A &amp; A Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T33" s="2" t="inlineStr">
@@ -2879,8 +2879,8 @@
       <c r="S34" s="2" t="inlineStr">
         <is>
           <t>Hi Neomis Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T34" s="2" t="inlineStr">
@@ -2942,8 +2942,8 @@
       <c r="S35" s="2" t="inlineStr">
         <is>
           <t>Hi Cheron Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T35" s="2" t="inlineStr">
@@ -3009,8 +3009,8 @@
       <c r="S36" s="2" t="inlineStr">
         <is>
           <t>Hi Samphire Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T36" s="2" t="inlineStr">
@@ -3076,8 +3076,8 @@
       <c r="S37" s="2" t="inlineStr">
         <is>
           <t>Hi Shri Salon team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T37" s="2" t="inlineStr">
@@ -3143,8 +3143,8 @@
       <c r="S38" s="2" t="inlineStr">
         <is>
           <t>Hi Manicure Goa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T38" s="2" t="inlineStr">
@@ -3210,8 +3210,8 @@
       <c r="S39" s="2" t="inlineStr">
         <is>
           <t>Hi Nails &amp; Lashes Goa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T39" s="2" t="inlineStr">
@@ -3273,8 +3273,8 @@
       <c r="S40" s="2" t="inlineStr">
         <is>
           <t>Hi The Nail Lounge team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T40" s="2" t="inlineStr">
@@ -3348,8 +3348,8 @@
       <c r="S41" s="2" t="inlineStr">
         <is>
           <t>Hi Anew Cosmetic &amp; Aesthetic Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T41" s="2" t="inlineStr">
@@ -3415,8 +3415,8 @@
       <c r="S42" s="2" t="inlineStr">
         <is>
           <t>Hi Warren Tricomi Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T42" s="2" t="inlineStr">
@@ -3478,8 +3478,8 @@
       <c r="S43" s="2" t="inlineStr">
         <is>
           <t>Hi The Bohem Salon &amp; Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T43" s="2" t="inlineStr">
@@ -3541,8 +3541,8 @@
       <c r="S44" s="2" t="inlineStr">
         <is>
           <t>Hi Royal Oak Spa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T44" s="2" t="inlineStr">
@@ -3604,8 +3604,8 @@
       <c r="S45" s="2" t="inlineStr">
         <is>
           <t>Hi Beyond Looks - A Complete Family Salon team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T45" s="2" t="inlineStr">
@@ -3667,8 +3667,8 @@
       <c r="S46" s="2" t="inlineStr">
         <is>
           <t>Hi Radiance Unisex Hair &amp; Beauty Salon team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
-It takes 10 minutes, in person or on a call, and everyone who takes part gets the full Goa findings report free. Could I drop by this Saturday, or would a quick call Mon-Wed be easier?
-If you're short on time, I can send a 2-minute form instead. Thank you!</t>
+It takes 10 minutes, in person or on a call. Could I drop by this week, or would a quick call be easier? If you're short on time, I can send a 2-minute form instead.
+As a thank-you, everyone who takes part gets the full Goa findings report free, plus a completely free trial of the small tool we're building from what we learn: 15 days, 20 days or a month, whichever suits you. Thank you!</t>
         </is>
       </c>
       <c r="T46" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Pipeline: mark 8 emailed leads as Messaged (26 Oct)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBvzkEqm3wQqXonEiSiA31
</commit_message>
<xml_diff>
--- a/2-pipeline/goa-leads-pipeline-v1.xlsx
+++ b/2-pipeline/goa-leads-pipeline-v1.xlsx
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1182,13 +1182,21 @@
           <t>https://physiotherapygoa.com</t>
         </is>
       </c>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
+      <c r="L9" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct.</t>
+        </is>
+      </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
           <t>Hi Physiotherapeautics team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1233,7 +1241,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1261,13 +1269,21 @@
           <t>https://physiofoxindia.com</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="L10" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
       <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct.</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
           <t>Hi PhysioFox: The Health Studio team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1312,7 +1328,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1340,13 +1356,21 @@
           <t>https://physioedgegoa.com</t>
         </is>
       </c>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="L11" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct.</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
           <t>Hi Physioedge Physiotherapy team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -3959,7 +3983,6 @@
           <t>SlotBack Goa discovery pipeline</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
Pipeline: add emails and Messaged stage for remaining 5 emailed leads
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBvzkEqm3wQqXonEiSiA31
</commit_message>
<xml_diff>
--- a/2-pipeline/goa-leads-pipeline-v1.xlsx
+++ b/2-pipeline/goa-leads-pipeline-v1.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -725,7 +725,11 @@
           <t>Open WhatsApp chat</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>aestheticdna.goa@gmail.com</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>@aestheticdna.goa</t>
@@ -736,13 +740,21 @@
           <t>https://aestheticdna.com</t>
         </is>
       </c>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
+      <c r="L3" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct to aestheticdna.goa@gmail.com.</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
           <t>Hi Aesthetic DNA team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1004,7 +1016,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1017,7 +1029,11 @@
           <t>Open WhatsApp chat</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>smilecraftgoa@gmail.com</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>@smilecraftgoa</t>
@@ -1028,13 +1044,21 @@
           <t>http://smilecraftgoa.com</t>
         </is>
       </c>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct to smilecraftgoa@gmail.com.</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>Hi Smile Craft Goa team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1079,7 +1103,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1092,7 +1116,11 @@
           <t>Open WhatsApp chat</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>connect@drnaiksdentalstudio.com</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>@drnaiksdentalstudio</t>
@@ -1103,13 +1131,21 @@
           <t>https://drnaiksdentalstudio.com</t>
         </is>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
+      <c r="L8" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct to connect@drnaiksdentalstudio.com.</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Hi Dr. Naik's Dental Studio / Kids-N-Braces team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1817,7 +1853,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1830,7 +1866,11 @@
           <t>Open WhatsApp chat</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>studio32india@gmail.com</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t>@studio32goa</t>
@@ -1841,13 +1881,21 @@
           <t>https://studio32india.com</t>
         </is>
       </c>
-      <c r="L18" s="5" t="n"/>
-      <c r="M18" s="5" t="n"/>
+      <c r="L18" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct to studio32india@gmail.com.</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
           <t>Hi Studio32 Dental team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.
@@ -1892,7 +1940,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Messaged</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1905,20 +1953,32 @@
           <t>Open WhatsApp chat</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>care@dremericodentalclinic.com</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>https://dremericodentalclinic.com</t>
         </is>
       </c>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
+      <c r="L19" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>46324</v>
+      </c>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
       <c r="Q19" s="2" t="n"/>
-      <c r="R19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Study email + free trial offer sent 26 Oct to care@dremericodentalclinic.com.</t>
+        </is>
+      </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
           <t>Hi Dr. Emerico's Dental Clinic team, I'm Atreya. I'm running a short study of pre-booked businesses in Goa (clinics, studios and salons) on how bookings, cancellations and no-shows affect the working day.

</xml_diff>

<commit_message>
Pipeline: note bounced and delayed study emails (28 Oct)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBvzkEqm3wQqXonEiSiA31
</commit_message>
<xml_diff>
--- a/2-pipeline/goa-leads-pipeline-v1.xlsx
+++ b/2-pipeline/goa-leads-pipeline-v1.xlsx
@@ -1143,7 +1143,7 @@
       <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Study email + free trial offer sent 26 Oct to connect@drnaiksdentalstudio.com.</t>
+          <t>Email delivery delayed 27 Oct (Gmail retrying). Call instead. Study email + free trial offer sent 26 Oct to connect@drnaiksdentalstudio.com.</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1317,7 +1317,7 @@
       <c r="Q10" s="2" t="n"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Study email + free trial offer sent 26 Oct.</t>
+          <t>EMAIL BOUNCED 26 Oct (server misconfigured). Call or WhatsApp instead. Study email + free trial offer sent 26 Oct.</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1976,7 +1976,7 @@
       <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Study email + free trial offer sent 26 Oct to care@dremericodentalclinic.com.</t>
+          <t>EMAIL BOUNCED 26 Oct (server misconfigured). Call instead. Study email + free trial offer sent 26 Oct to care@dremericodentalclinic.com.</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">

</xml_diff>